<commit_message>
Update bilingual interface, distributions, session management and verification
</commit_message>
<xml_diff>
--- a/project_risk_template_v2_2.xlsx
+++ b/project_risk_template_v2_2.xlsx
@@ -29,7 +29,7 @@
   <definedNames>
     <definedName name="RiskCategoryOptions">Risk_Categories!$A$3:$A$20</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" calcMode="auto" fullCalcOnLoad="1" forceFullCalc="1"/>
   <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -2348,7 +2348,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="63">
+  <cellXfs count="72">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -2520,6 +2520,33 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -4256,7 +4283,7 @@
     <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Duration_Max" dataDxfId="39"/>
     <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="Duration_Mean" dataDxfId="38"/>
     <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="Duration_SD" dataDxfId="37"/>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="Base_Cost" dataDxfId="36"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="Fixed_Cost" dataDxfId="36"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -4526,7 +4553,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H41"/>
+  <dimension ref="A1:H47"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="24" style="12" customWidth="1"/>
@@ -4864,6 +4891,78 @@
       </c>
       <c r="B41" s="3" t="s">
         <v>80</v>
+      </c>
+    </row>
+    <row r="42" ht="75" customHeight="1">
+      <c r="A42" s="70" t="inlineStr">
+        <is>
+          <t>Distribution parameters</t>
+        </is>
+      </c>
+      <c r="B42" s="71" t="inlineStr">
+        <is>
+          <t>Required parameter cells are highlighted for the selected distribution; unused cells remain neutral and their existing contents are retained.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="75" customHeight="1">
+      <c r="A43" s="70" t="inlineStr">
+        <is>
+          <t>Exponential</t>
+        </is>
+      </c>
+      <c r="B43" s="71" t="inlineStr">
+        <is>
+          <t>Enter an arithmetic Mean &gt; 0. Standard deviation and three-point fields are unused. The distribution is nonnegative and has no finite maximum.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="75" customHeight="1">
+      <c r="A44" s="70" t="inlineStr">
+        <is>
+          <t>Lognormal and Gamma</t>
+        </is>
+      </c>
+      <c r="B44" s="71" t="inlineStr">
+        <is>
+          <t>Enter arithmetic Mean &gt; 0 and Standard deviation &gt; 0 in the original units. Logarithmic parameters and Gamma shape/scale are derived internally. No finite maximum is imposed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="75" customHeight="1">
+      <c r="A45" s="70" t="inlineStr">
+        <is>
+          <t>Optional cost distributions</t>
+        </is>
+      </c>
+      <c r="B45" s="71" t="inlineStr">
+        <is>
+          <t>Leave Cost_Model blank to retain the linked Fixed_Cost workflow. An explicit cost model uses its highlighted Cost_* parameters for the duration-independent component; the existing duration rate and direct risk costs still apply.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="75" customHeight="1">
+      <c r="A46" s="70" t="inlineStr">
+        <is>
+          <t>Distribution scope</t>
+        </is>
+      </c>
+      <c r="B46" s="71" t="inlineStr">
+        <is>
+          <t>These choices describe activity durations, intrinsic activity costs and mapped impact magnitudes. Risk occurrence probabilities retain their original Fixed/Uniform support.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="75" customHeight="1">
+      <c r="A47" s="70" t="inlineStr">
+        <is>
+          <t>Reference mean</t>
+        </is>
+      </c>
+      <c r="B47" s="71" t="inlineStr">
+        <is>
+          <t>Reference CPM and linked cost-rate formulas use the entered arithmetic Mean for Exponential, Lognormal and Gamma. Recalculate and save after edits before uploading.</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -6093,7 +6192,7 @@
         <v>12000</v>
       </c>
       <c r="C3" s="49">
-        <f>IF(Activities!D3="Fixed",Activities!E3,IF(Activities!D3="Triangular",(Activities!F3+Activities!G3+Activities!H3)/3,IF(Activities!D3="Beta-PERT",(Activities!F3+4*Activities!G3+Activities!H3)/6,IF(Activities!D3="Normal",Activities!I3,IF(Activities!D3="Uniform",(Activities!F3+Activities!H3)/2,NA())))))</f>
+        <f>IF(Activities!D3="Fixed",Activities!E3,IF(Activities!D3="Triangular",(Activities!F3+Activities!G3+Activities!H3)/3,IF(Activities!D3="Beta-PERT",(Activities!F3+4*Activities!G3+Activities!H3)/6,IF(Activities!D3="Normal",Activities!I3,IF(Activities!D3="Uniform",(Activities!F3+Activities!H3)/2,IF(OR(Activities!D3="Exponential",Activities!D3="Lognormal",Activities!D3="Gamma"),Activities!I3,NA()))))))</f>
         <v>3</v>
       </c>
       <c r="D3" s="50">
@@ -6127,7 +6226,7 @@
         <v>8000</v>
       </c>
       <c r="C4" s="49">
-        <f>IF(Activities!D4="Fixed",Activities!E4,IF(Activities!D4="Triangular",(Activities!F4+Activities!G4+Activities!H4)/3,IF(Activities!D4="Beta-PERT",(Activities!F4+4*Activities!G4+Activities!H4)/6,IF(Activities!D4="Normal",Activities!I4,IF(Activities!D4="Uniform",(Activities!F4+Activities!H4)/2,NA())))))</f>
+        <f>IF(Activities!D4="Fixed",Activities!E4,IF(Activities!D4="Triangular",(Activities!F4+Activities!G4+Activities!H4)/3,IF(Activities!D4="Beta-PERT",(Activities!F4+4*Activities!G4+Activities!H4)/6,IF(Activities!D4="Normal",Activities!I4,IF(Activities!D4="Uniform",(Activities!F4+Activities!H4)/2,IF(OR(Activities!D4="Exponential",Activities!D4="Lognormal",Activities!D4="Gamma"),Activities!I4,NA()))))))</f>
         <v>3.3333333333333335</v>
       </c>
       <c r="D4" s="50">
@@ -6161,7 +6260,7 @@
         <v>25000</v>
       </c>
       <c r="C5" s="49">
-        <f>IF(Activities!D5="Fixed",Activities!E5,IF(Activities!D5="Triangular",(Activities!F5+Activities!G5+Activities!H5)/3,IF(Activities!D5="Beta-PERT",(Activities!F5+4*Activities!G5+Activities!H5)/6,IF(Activities!D5="Normal",Activities!I5,IF(Activities!D5="Uniform",(Activities!F5+Activities!H5)/2,NA())))))</f>
+        <f>IF(Activities!D5="Fixed",Activities!E5,IF(Activities!D5="Triangular",(Activities!F5+Activities!G5+Activities!H5)/3,IF(Activities!D5="Beta-PERT",(Activities!F5+4*Activities!G5+Activities!H5)/6,IF(Activities!D5="Normal",Activities!I5,IF(Activities!D5="Uniform",(Activities!F5+Activities!H5)/2,IF(OR(Activities!D5="Exponential",Activities!D5="Lognormal",Activities!D5="Gamma"),Activities!I5,NA()))))))</f>
         <v>6.166666666666667</v>
       </c>
       <c r="D5" s="50">
@@ -6195,7 +6294,7 @@
         <v>18000</v>
       </c>
       <c r="C6" s="49">
-        <f>IF(Activities!D6="Fixed",Activities!E6,IF(Activities!D6="Triangular",(Activities!F6+Activities!G6+Activities!H6)/3,IF(Activities!D6="Beta-PERT",(Activities!F6+4*Activities!G6+Activities!H6)/6,IF(Activities!D6="Normal",Activities!I6,IF(Activities!D6="Uniform",(Activities!F6+Activities!H6)/2,NA())))))</f>
+        <f>IF(Activities!D6="Fixed",Activities!E6,IF(Activities!D6="Triangular",(Activities!F6+Activities!G6+Activities!H6)/3,IF(Activities!D6="Beta-PERT",(Activities!F6+4*Activities!G6+Activities!H6)/6,IF(Activities!D6="Normal",Activities!I6,IF(Activities!D6="Uniform",(Activities!F6+Activities!H6)/2,IF(OR(Activities!D6="Exponential",Activities!D6="Lognormal",Activities!D6="Gamma"),Activities!I6,NA()))))))</f>
         <v>5</v>
       </c>
       <c r="D6" s="50">
@@ -6229,7 +6328,7 @@
         <v>65000</v>
       </c>
       <c r="C7" s="49">
-        <f>IF(Activities!D7="Fixed",Activities!E7,IF(Activities!D7="Triangular",(Activities!F7+Activities!G7+Activities!H7)/3,IF(Activities!D7="Beta-PERT",(Activities!F7+4*Activities!G7+Activities!H7)/6,IF(Activities!D7="Normal",Activities!I7,IF(Activities!D7="Uniform",(Activities!F7+Activities!H7)/2,NA())))))</f>
+        <f>IF(Activities!D7="Fixed",Activities!E7,IF(Activities!D7="Triangular",(Activities!F7+Activities!G7+Activities!H7)/3,IF(Activities!D7="Beta-PERT",(Activities!F7+4*Activities!G7+Activities!H7)/6,IF(Activities!D7="Normal",Activities!I7,IF(Activities!D7="Uniform",(Activities!F7+Activities!H7)/2,IF(OR(Activities!D7="Exponential",Activities!D7="Lognormal",Activities!D7="Gamma"),Activities!I7,NA()))))))</f>
         <v>10</v>
       </c>
       <c r="D7" s="50">
@@ -6263,7 +6362,7 @@
         <v>38000</v>
       </c>
       <c r="C8" s="49">
-        <f>IF(Activities!D8="Fixed",Activities!E8,IF(Activities!D8="Triangular",(Activities!F8+Activities!G8+Activities!H8)/3,IF(Activities!D8="Beta-PERT",(Activities!F8+4*Activities!G8+Activities!H8)/6,IF(Activities!D8="Normal",Activities!I8,IF(Activities!D8="Uniform",(Activities!F8+Activities!H8)/2,NA())))))</f>
+        <f>IF(Activities!D8="Fixed",Activities!E8,IF(Activities!D8="Triangular",(Activities!F8+Activities!G8+Activities!H8)/3,IF(Activities!D8="Beta-PERT",(Activities!F8+4*Activities!G8+Activities!H8)/6,IF(Activities!D8="Normal",Activities!I8,IF(Activities!D8="Uniform",(Activities!F8+Activities!H8)/2,IF(OR(Activities!D8="Exponential",Activities!D8="Lognormal",Activities!D8="Gamma"),Activities!I8,NA()))))))</f>
         <v>6.333333333333333</v>
       </c>
       <c r="D8" s="50">
@@ -6297,7 +6396,7 @@
         <v>85000</v>
       </c>
       <c r="C9" s="49">
-        <f>IF(Activities!D9="Fixed",Activities!E9,IF(Activities!D9="Triangular",(Activities!F9+Activities!G9+Activities!H9)/3,IF(Activities!D9="Beta-PERT",(Activities!F9+4*Activities!G9+Activities!H9)/6,IF(Activities!D9="Normal",Activities!I9,IF(Activities!D9="Uniform",(Activities!F9+Activities!H9)/2,NA())))))</f>
+        <f>IF(Activities!D9="Fixed",Activities!E9,IF(Activities!D9="Triangular",(Activities!F9+Activities!G9+Activities!H9)/3,IF(Activities!D9="Beta-PERT",(Activities!F9+4*Activities!G9+Activities!H9)/6,IF(Activities!D9="Normal",Activities!I9,IF(Activities!D9="Uniform",(Activities!F9+Activities!H9)/2,IF(OR(Activities!D9="Exponential",Activities!D9="Lognormal",Activities!D9="Gamma"),Activities!I9,NA()))))))</f>
         <v>12.166666666666666</v>
       </c>
       <c r="D9" s="50">
@@ -6331,7 +6430,7 @@
         <v>82000</v>
       </c>
       <c r="C10" s="49">
-        <f>IF(Activities!D10="Fixed",Activities!E10,IF(Activities!D10="Triangular",(Activities!F10+Activities!G10+Activities!H10)/3,IF(Activities!D10="Beta-PERT",(Activities!F10+4*Activities!G10+Activities!H10)/6,IF(Activities!D10="Normal",Activities!I10,IF(Activities!D10="Uniform",(Activities!F10+Activities!H10)/2,NA())))))</f>
+        <f>IF(Activities!D10="Fixed",Activities!E10,IF(Activities!D10="Triangular",(Activities!F10+Activities!G10+Activities!H10)/3,IF(Activities!D10="Beta-PERT",(Activities!F10+4*Activities!G10+Activities!H10)/6,IF(Activities!D10="Normal",Activities!I10,IF(Activities!D10="Uniform",(Activities!F10+Activities!H10)/2,IF(OR(Activities!D10="Exponential",Activities!D10="Lognormal",Activities!D10="Gamma"),Activities!I10,NA()))))))</f>
         <v>11</v>
       </c>
       <c r="D10" s="50">
@@ -6365,7 +6464,7 @@
         <v>42000</v>
       </c>
       <c r="C11" s="49">
-        <f>IF(Activities!D11="Fixed",Activities!E11,IF(Activities!D11="Triangular",(Activities!F11+Activities!G11+Activities!H11)/3,IF(Activities!D11="Beta-PERT",(Activities!F11+4*Activities!G11+Activities!H11)/6,IF(Activities!D11="Normal",Activities!I11,IF(Activities!D11="Uniform",(Activities!F11+Activities!H11)/2,NA())))))</f>
+        <f>IF(Activities!D11="Fixed",Activities!E11,IF(Activities!D11="Triangular",(Activities!F11+Activities!G11+Activities!H11)/3,IF(Activities!D11="Beta-PERT",(Activities!F11+4*Activities!G11+Activities!H11)/6,IF(Activities!D11="Normal",Activities!I11,IF(Activities!D11="Uniform",(Activities!F11+Activities!H11)/2,IF(OR(Activities!D11="Exponential",Activities!D11="Lognormal",Activities!D11="Gamma"),Activities!I11,NA()))))))</f>
         <v>7</v>
       </c>
       <c r="D11" s="50">
@@ -6399,7 +6498,7 @@
         <v>50000</v>
       </c>
       <c r="C12" s="49">
-        <f>IF(Activities!D12="Fixed",Activities!E12,IF(Activities!D12="Triangular",(Activities!F12+Activities!G12+Activities!H12)/3,IF(Activities!D12="Beta-PERT",(Activities!F12+4*Activities!G12+Activities!H12)/6,IF(Activities!D12="Normal",Activities!I12,IF(Activities!D12="Uniform",(Activities!F12+Activities!H12)/2,NA())))))</f>
+        <f>IF(Activities!D12="Fixed",Activities!E12,IF(Activities!D12="Triangular",(Activities!F12+Activities!G12+Activities!H12)/3,IF(Activities!D12="Beta-PERT",(Activities!F12+4*Activities!G12+Activities!H12)/6,IF(Activities!D12="Normal",Activities!I12,IF(Activities!D12="Uniform",(Activities!F12+Activities!H12)/2,IF(OR(Activities!D12="Exponential",Activities!D12="Lognormal",Activities!D12="Gamma"),Activities!I12,NA()))))))</f>
         <v>10.666666666666666</v>
       </c>
       <c r="D12" s="50">
@@ -6433,7 +6532,7 @@
         <v>32000</v>
       </c>
       <c r="C13" s="49">
-        <f>IF(Activities!D13="Fixed",Activities!E13,IF(Activities!D13="Triangular",(Activities!F13+Activities!G13+Activities!H13)/3,IF(Activities!D13="Beta-PERT",(Activities!F13+4*Activities!G13+Activities!H13)/6,IF(Activities!D13="Normal",Activities!I13,IF(Activities!D13="Uniform",(Activities!F13+Activities!H13)/2,NA())))))</f>
+        <f>IF(Activities!D13="Fixed",Activities!E13,IF(Activities!D13="Triangular",(Activities!F13+Activities!G13+Activities!H13)/3,IF(Activities!D13="Beta-PERT",(Activities!F13+4*Activities!G13+Activities!H13)/6,IF(Activities!D13="Normal",Activities!I13,IF(Activities!D13="Uniform",(Activities!F13+Activities!H13)/2,IF(OR(Activities!D13="Exponential",Activities!D13="Lognormal",Activities!D13="Gamma"),Activities!I13,NA()))))))</f>
         <v>8.3333333333333339</v>
       </c>
       <c r="D13" s="50">
@@ -6467,7 +6566,7 @@
         <v>35000</v>
       </c>
       <c r="C14" s="49">
-        <f>IF(Activities!D14="Fixed",Activities!E14,IF(Activities!D14="Triangular",(Activities!F14+Activities!G14+Activities!H14)/3,IF(Activities!D14="Beta-PERT",(Activities!F14+4*Activities!G14+Activities!H14)/6,IF(Activities!D14="Normal",Activities!I14,IF(Activities!D14="Uniform",(Activities!F14+Activities!H14)/2,NA())))))</f>
+        <f>IF(Activities!D14="Fixed",Activities!E14,IF(Activities!D14="Triangular",(Activities!F14+Activities!G14+Activities!H14)/3,IF(Activities!D14="Beta-PERT",(Activities!F14+4*Activities!G14+Activities!H14)/6,IF(Activities!D14="Normal",Activities!I14,IF(Activities!D14="Uniform",(Activities!F14+Activities!H14)/2,IF(OR(Activities!D14="Exponential",Activities!D14="Lognormal",Activities!D14="Gamma"),Activities!I14,NA()))))))</f>
         <v>8</v>
       </c>
       <c r="D14" s="50">
@@ -6501,7 +6600,7 @@
         <v>36000</v>
       </c>
       <c r="C15" s="49">
-        <f>IF(Activities!D15="Fixed",Activities!E15,IF(Activities!D15="Triangular",(Activities!F15+Activities!G15+Activities!H15)/3,IF(Activities!D15="Beta-PERT",(Activities!F15+4*Activities!G15+Activities!H15)/6,IF(Activities!D15="Normal",Activities!I15,IF(Activities!D15="Uniform",(Activities!F15+Activities!H15)/2,NA())))))</f>
+        <f>IF(Activities!D15="Fixed",Activities!E15,IF(Activities!D15="Triangular",(Activities!F15+Activities!G15+Activities!H15)/3,IF(Activities!D15="Beta-PERT",(Activities!F15+4*Activities!G15+Activities!H15)/6,IF(Activities!D15="Normal",Activities!I15,IF(Activities!D15="Uniform",(Activities!F15+Activities!H15)/2,IF(OR(Activities!D15="Exponential",Activities!D15="Lognormal",Activities!D15="Gamma"),Activities!I15,NA()))))))</f>
         <v>8</v>
       </c>
       <c r="D15" s="50">
@@ -6535,7 +6634,7 @@
         <v>28000</v>
       </c>
       <c r="C16" s="49">
-        <f>IF(Activities!D16="Fixed",Activities!E16,IF(Activities!D16="Triangular",(Activities!F16+Activities!G16+Activities!H16)/3,IF(Activities!D16="Beta-PERT",(Activities!F16+4*Activities!G16+Activities!H16)/6,IF(Activities!D16="Normal",Activities!I16,IF(Activities!D16="Uniform",(Activities!F16+Activities!H16)/2,NA())))))</f>
+        <f>IF(Activities!D16="Fixed",Activities!E16,IF(Activities!D16="Triangular",(Activities!F16+Activities!G16+Activities!H16)/3,IF(Activities!D16="Beta-PERT",(Activities!F16+4*Activities!G16+Activities!H16)/6,IF(Activities!D16="Normal",Activities!I16,IF(Activities!D16="Uniform",(Activities!F16+Activities!H16)/2,IF(OR(Activities!D16="Exponential",Activities!D16="Lognormal",Activities!D16="Gamma"),Activities!I16,NA()))))))</f>
         <v>6.666666666666667</v>
       </c>
       <c r="D16" s="50">
@@ -6569,7 +6668,7 @@
         <v>45000</v>
       </c>
       <c r="C17" s="49">
-        <f>IF(Activities!D17="Fixed",Activities!E17,IF(Activities!D17="Triangular",(Activities!F17+Activities!G17+Activities!H17)/3,IF(Activities!D17="Beta-PERT",(Activities!F17+4*Activities!G17+Activities!H17)/6,IF(Activities!D17="Normal",Activities!I17,IF(Activities!D17="Uniform",(Activities!F17+Activities!H17)/2,NA())))))</f>
+        <f>IF(Activities!D17="Fixed",Activities!E17,IF(Activities!D17="Triangular",(Activities!F17+Activities!G17+Activities!H17)/3,IF(Activities!D17="Beta-PERT",(Activities!F17+4*Activities!G17+Activities!H17)/6,IF(Activities!D17="Normal",Activities!I17,IF(Activities!D17="Uniform",(Activities!F17+Activities!H17)/2,IF(OR(Activities!D17="Exponential",Activities!D17="Lognormal",Activities!D17="Gamma"),Activities!I17,NA()))))))</f>
         <v>6.333333333333333</v>
       </c>
       <c r="D17" s="50">
@@ -6603,7 +6702,7 @@
         <v>22000</v>
       </c>
       <c r="C18" s="49">
-        <f>IF(Activities!D18="Fixed",Activities!E18,IF(Activities!D18="Triangular",(Activities!F18+Activities!G18+Activities!H18)/3,IF(Activities!D18="Beta-PERT",(Activities!F18+4*Activities!G18+Activities!H18)/6,IF(Activities!D18="Normal",Activities!I18,IF(Activities!D18="Uniform",(Activities!F18+Activities!H18)/2,NA())))))</f>
+        <f>IF(Activities!D18="Fixed",Activities!E18,IF(Activities!D18="Triangular",(Activities!F18+Activities!G18+Activities!H18)/3,IF(Activities!D18="Beta-PERT",(Activities!F18+4*Activities!G18+Activities!H18)/6,IF(Activities!D18="Normal",Activities!I18,IF(Activities!D18="Uniform",(Activities!F18+Activities!H18)/2,IF(OR(Activities!D18="Exponential",Activities!D18="Lognormal",Activities!D18="Gamma"),Activities!I18,NA()))))))</f>
         <v>5</v>
       </c>
       <c r="D18" s="50">
@@ -6637,7 +6736,7 @@
         <v>40000</v>
       </c>
       <c r="C19" s="49">
-        <f>IF(Activities!D19="Fixed",Activities!E19,IF(Activities!D19="Triangular",(Activities!F19+Activities!G19+Activities!H19)/3,IF(Activities!D19="Beta-PERT",(Activities!F19+4*Activities!G19+Activities!H19)/6,IF(Activities!D19="Normal",Activities!I19,IF(Activities!D19="Uniform",(Activities!F19+Activities!H19)/2,NA())))))</f>
+        <f>IF(Activities!D19="Fixed",Activities!E19,IF(Activities!D19="Triangular",(Activities!F19+Activities!G19+Activities!H19)/3,IF(Activities!D19="Beta-PERT",(Activities!F19+4*Activities!G19+Activities!H19)/6,IF(Activities!D19="Normal",Activities!I19,IF(Activities!D19="Uniform",(Activities!F19+Activities!H19)/2,IF(OR(Activities!D19="Exponential",Activities!D19="Lognormal",Activities!D19="Gamma"),Activities!I19,NA()))))))</f>
         <v>9</v>
       </c>
       <c r="D19" s="50">
@@ -6671,7 +6770,7 @@
         <v>48000</v>
       </c>
       <c r="C20" s="49">
-        <f>IF(Activities!D20="Fixed",Activities!E20,IF(Activities!D20="Triangular",(Activities!F20+Activities!G20+Activities!H20)/3,IF(Activities!D20="Beta-PERT",(Activities!F20+4*Activities!G20+Activities!H20)/6,IF(Activities!D20="Normal",Activities!I20,IF(Activities!D20="Uniform",(Activities!F20+Activities!H20)/2,NA())))))</f>
+        <f>IF(Activities!D20="Fixed",Activities!E20,IF(Activities!D20="Triangular",(Activities!F20+Activities!G20+Activities!H20)/3,IF(Activities!D20="Beta-PERT",(Activities!F20+4*Activities!G20+Activities!H20)/6,IF(Activities!D20="Normal",Activities!I20,IF(Activities!D20="Uniform",(Activities!F20+Activities!H20)/2,IF(OR(Activities!D20="Exponential",Activities!D20="Lognormal",Activities!D20="Gamma"),Activities!I20,NA()))))))</f>
         <v>9.6666666666666661</v>
       </c>
       <c r="D20" s="50">
@@ -6705,7 +6804,7 @@
         <v>52000</v>
       </c>
       <c r="C21" s="49">
-        <f>IF(Activities!D21="Fixed",Activities!E21,IF(Activities!D21="Triangular",(Activities!F21+Activities!G21+Activities!H21)/3,IF(Activities!D21="Beta-PERT",(Activities!F21+4*Activities!G21+Activities!H21)/6,IF(Activities!D21="Normal",Activities!I21,IF(Activities!D21="Uniform",(Activities!F21+Activities!H21)/2,NA())))))</f>
+        <f>IF(Activities!D21="Fixed",Activities!E21,IF(Activities!D21="Triangular",(Activities!F21+Activities!G21+Activities!H21)/3,IF(Activities!D21="Beta-PERT",(Activities!F21+4*Activities!G21+Activities!H21)/6,IF(Activities!D21="Normal",Activities!I21,IF(Activities!D21="Uniform",(Activities!F21+Activities!H21)/2,IF(OR(Activities!D21="Exponential",Activities!D21="Lognormal",Activities!D21="Gamma"),Activities!I21,NA()))))))</f>
         <v>9.1666666666666661</v>
       </c>
       <c r="D21" s="50">
@@ -6739,7 +6838,7 @@
         <v>26000</v>
       </c>
       <c r="C22" s="49">
-        <f>IF(Activities!D22="Fixed",Activities!E22,IF(Activities!D22="Triangular",(Activities!F22+Activities!G22+Activities!H22)/3,IF(Activities!D22="Beta-PERT",(Activities!F22+4*Activities!G22+Activities!H22)/6,IF(Activities!D22="Normal",Activities!I22,IF(Activities!D22="Uniform",(Activities!F22+Activities!H22)/2,NA())))))</f>
+        <f>IF(Activities!D22="Fixed",Activities!E22,IF(Activities!D22="Triangular",(Activities!F22+Activities!G22+Activities!H22)/3,IF(Activities!D22="Beta-PERT",(Activities!F22+4*Activities!G22+Activities!H22)/6,IF(Activities!D22="Normal",Activities!I22,IF(Activities!D22="Uniform",(Activities!F22+Activities!H22)/2,IF(OR(Activities!D22="Exponential",Activities!D22="Lognormal",Activities!D22="Gamma"),Activities!I22,NA()))))))</f>
         <v>6</v>
       </c>
       <c r="D22" s="50">
@@ -6773,7 +6872,7 @@
         <v>38000</v>
       </c>
       <c r="C23" s="49">
-        <f>IF(Activities!D23="Fixed",Activities!E23,IF(Activities!D23="Triangular",(Activities!F23+Activities!G23+Activities!H23)/3,IF(Activities!D23="Beta-PERT",(Activities!F23+4*Activities!G23+Activities!H23)/6,IF(Activities!D23="Normal",Activities!I23,IF(Activities!D23="Uniform",(Activities!F23+Activities!H23)/2,NA())))))</f>
+        <f>IF(Activities!D23="Fixed",Activities!E23,IF(Activities!D23="Triangular",(Activities!F23+Activities!G23+Activities!H23)/3,IF(Activities!D23="Beta-PERT",(Activities!F23+4*Activities!G23+Activities!H23)/6,IF(Activities!D23="Normal",Activities!I23,IF(Activities!D23="Uniform",(Activities!F23+Activities!H23)/2,IF(OR(Activities!D23="Exponential",Activities!D23="Lognormal",Activities!D23="Gamma"),Activities!I23,NA()))))))</f>
         <v>9</v>
       </c>
       <c r="D23" s="50">
@@ -6807,7 +6906,7 @@
         <v>30000</v>
       </c>
       <c r="C24" s="49">
-        <f>IF(Activities!D24="Fixed",Activities!E24,IF(Activities!D24="Triangular",(Activities!F24+Activities!G24+Activities!H24)/3,IF(Activities!D24="Beta-PERT",(Activities!F24+4*Activities!G24+Activities!H24)/6,IF(Activities!D24="Normal",Activities!I24,IF(Activities!D24="Uniform",(Activities!F24+Activities!H24)/2,NA())))))</f>
+        <f>IF(Activities!D24="Fixed",Activities!E24,IF(Activities!D24="Triangular",(Activities!F24+Activities!G24+Activities!H24)/3,IF(Activities!D24="Beta-PERT",(Activities!F24+4*Activities!G24+Activities!H24)/6,IF(Activities!D24="Normal",Activities!I24,IF(Activities!D24="Uniform",(Activities!F24+Activities!H24)/2,IF(OR(Activities!D24="Exponential",Activities!D24="Lognormal",Activities!D24="Gamma"),Activities!I24,NA()))))))</f>
         <v>6.333333333333333</v>
       </c>
       <c r="D24" s="50">
@@ -6841,7 +6940,7 @@
         <v>32000</v>
       </c>
       <c r="C25" s="49">
-        <f>IF(Activities!D25="Fixed",Activities!E25,IF(Activities!D25="Triangular",(Activities!F25+Activities!G25+Activities!H25)/3,IF(Activities!D25="Beta-PERT",(Activities!F25+4*Activities!G25+Activities!H25)/6,IF(Activities!D25="Normal",Activities!I25,IF(Activities!D25="Uniform",(Activities!F25+Activities!H25)/2,NA())))))</f>
+        <f>IF(Activities!D25="Fixed",Activities!E25,IF(Activities!D25="Triangular",(Activities!F25+Activities!G25+Activities!H25)/3,IF(Activities!D25="Beta-PERT",(Activities!F25+4*Activities!G25+Activities!H25)/6,IF(Activities!D25="Normal",Activities!I25,IF(Activities!D25="Uniform",(Activities!F25+Activities!H25)/2,IF(OR(Activities!D25="Exponential",Activities!D25="Lognormal",Activities!D25="Gamma"),Activities!I25,NA()))))))</f>
         <v>6.166666666666667</v>
       </c>
       <c r="D25" s="50">
@@ -6875,7 +6974,7 @@
         <v>42000</v>
       </c>
       <c r="C26" s="49">
-        <f>IF(Activities!D26="Fixed",Activities!E26,IF(Activities!D26="Triangular",(Activities!F26+Activities!G26+Activities!H26)/3,IF(Activities!D26="Beta-PERT",(Activities!F26+4*Activities!G26+Activities!H26)/6,IF(Activities!D26="Normal",Activities!I26,IF(Activities!D26="Uniform",(Activities!F26+Activities!H26)/2,NA())))))</f>
+        <f>IF(Activities!D26="Fixed",Activities!E26,IF(Activities!D26="Triangular",(Activities!F26+Activities!G26+Activities!H26)/3,IF(Activities!D26="Beta-PERT",(Activities!F26+4*Activities!G26+Activities!H26)/6,IF(Activities!D26="Normal",Activities!I26,IF(Activities!D26="Uniform",(Activities!F26+Activities!H26)/2,IF(OR(Activities!D26="Exponential",Activities!D26="Lognormal",Activities!D26="Gamma"),Activities!I26,NA()))))))</f>
         <v>8</v>
       </c>
       <c r="D26" s="50">
@@ -6909,7 +7008,7 @@
         <v>55000</v>
       </c>
       <c r="C27" s="49">
-        <f>IF(Activities!D27="Fixed",Activities!E27,IF(Activities!D27="Triangular",(Activities!F27+Activities!G27+Activities!H27)/3,IF(Activities!D27="Beta-PERT",(Activities!F27+4*Activities!G27+Activities!H27)/6,IF(Activities!D27="Normal",Activities!I27,IF(Activities!D27="Uniform",(Activities!F27+Activities!H27)/2,NA())))))</f>
+        <f>IF(Activities!D27="Fixed",Activities!E27,IF(Activities!D27="Triangular",(Activities!F27+Activities!G27+Activities!H27)/3,IF(Activities!D27="Beta-PERT",(Activities!F27+4*Activities!G27+Activities!H27)/6,IF(Activities!D27="Normal",Activities!I27,IF(Activities!D27="Uniform",(Activities!F27+Activities!H27)/2,IF(OR(Activities!D27="Exponential",Activities!D27="Lognormal",Activities!D27="Gamma"),Activities!I27,NA()))))))</f>
         <v>9</v>
       </c>
       <c r="D27" s="50">
@@ -6943,7 +7042,7 @@
         <v>18000</v>
       </c>
       <c r="C28" s="49">
-        <f>IF(Activities!D28="Fixed",Activities!E28,IF(Activities!D28="Triangular",(Activities!F28+Activities!G28+Activities!H28)/3,IF(Activities!D28="Beta-PERT",(Activities!F28+4*Activities!G28+Activities!H28)/6,IF(Activities!D28="Normal",Activities!I28,IF(Activities!D28="Uniform",(Activities!F28+Activities!H28)/2,NA())))))</f>
+        <f>IF(Activities!D28="Fixed",Activities!E28,IF(Activities!D28="Triangular",(Activities!F28+Activities!G28+Activities!H28)/3,IF(Activities!D28="Beta-PERT",(Activities!F28+4*Activities!G28+Activities!H28)/6,IF(Activities!D28="Normal",Activities!I28,IF(Activities!D28="Uniform",(Activities!F28+Activities!H28)/2,IF(OR(Activities!D28="Exponential",Activities!D28="Lognormal",Activities!D28="Gamma"),Activities!I28,NA()))))))</f>
         <v>5.333333333333333</v>
       </c>
       <c r="D28" s="50">
@@ -6977,7 +7076,7 @@
         <v>20000</v>
       </c>
       <c r="C29" s="49">
-        <f>IF(Activities!D29="Fixed",Activities!E29,IF(Activities!D29="Triangular",(Activities!F29+Activities!G29+Activities!H29)/3,IF(Activities!D29="Beta-PERT",(Activities!F29+4*Activities!G29+Activities!H29)/6,IF(Activities!D29="Normal",Activities!I29,IF(Activities!D29="Uniform",(Activities!F29+Activities!H29)/2,NA())))))</f>
+        <f>IF(Activities!D29="Fixed",Activities!E29,IF(Activities!D29="Triangular",(Activities!F29+Activities!G29+Activities!H29)/3,IF(Activities!D29="Beta-PERT",(Activities!F29+4*Activities!G29+Activities!H29)/6,IF(Activities!D29="Normal",Activities!I29,IF(Activities!D29="Uniform",(Activities!F29+Activities!H29)/2,IF(OR(Activities!D29="Exponential",Activities!D29="Lognormal",Activities!D29="Gamma"),Activities!I29,NA()))))))</f>
         <v>6.333333333333333</v>
       </c>
       <c r="D29" s="50">
@@ -7011,7 +7110,7 @@
         <v>15000</v>
       </c>
       <c r="C30" s="49">
-        <f>IF(Activities!D30="Fixed",Activities!E30,IF(Activities!D30="Triangular",(Activities!F30+Activities!G30+Activities!H30)/3,IF(Activities!D30="Beta-PERT",(Activities!F30+4*Activities!G30+Activities!H30)/6,IF(Activities!D30="Normal",Activities!I30,IF(Activities!D30="Uniform",(Activities!F30+Activities!H30)/2,NA())))))</f>
+        <f>IF(Activities!D30="Fixed",Activities!E30,IF(Activities!D30="Triangular",(Activities!F30+Activities!G30+Activities!H30)/3,IF(Activities!D30="Beta-PERT",(Activities!F30+4*Activities!G30+Activities!H30)/6,IF(Activities!D30="Normal",Activities!I30,IF(Activities!D30="Uniform",(Activities!F30+Activities!H30)/2,IF(OR(Activities!D30="Exponential",Activities!D30="Lognormal",Activities!D30="Gamma"),Activities!I30,NA()))))))</f>
         <v>5</v>
       </c>
       <c r="D30" s="50">
@@ -7045,7 +7144,7 @@
         <v>10000</v>
       </c>
       <c r="C31" s="49">
-        <f>IF(Activities!D31="Fixed",Activities!E31,IF(Activities!D31="Triangular",(Activities!F31+Activities!G31+Activities!H31)/3,IF(Activities!D31="Beta-PERT",(Activities!F31+4*Activities!G31+Activities!H31)/6,IF(Activities!D31="Normal",Activities!I31,IF(Activities!D31="Uniform",(Activities!F31+Activities!H31)/2,NA())))))</f>
+        <f>IF(Activities!D31="Fixed",Activities!E31,IF(Activities!D31="Triangular",(Activities!F31+Activities!G31+Activities!H31)/3,IF(Activities!D31="Beta-PERT",(Activities!F31+4*Activities!G31+Activities!H31)/6,IF(Activities!D31="Normal",Activities!I31,IF(Activities!D31="Uniform",(Activities!F31+Activities!H31)/2,IF(OR(Activities!D31="Exponential",Activities!D31="Lognormal",Activities!D31="Gamma"),Activities!I31,NA()))))))</f>
         <v>4.333333333333333</v>
       </c>
       <c r="D31" s="50">
@@ -7079,7 +7178,7 @@
         <v>8000</v>
       </c>
       <c r="C32" s="49">
-        <f>IF(Activities!D32="Fixed",Activities!E32,IF(Activities!D32="Triangular",(Activities!F32+Activities!G32+Activities!H32)/3,IF(Activities!D32="Beta-PERT",(Activities!F32+4*Activities!G32+Activities!H32)/6,IF(Activities!D32="Normal",Activities!I32,IF(Activities!D32="Uniform",(Activities!F32+Activities!H32)/2,NA())))))</f>
+        <f>IF(Activities!D32="Fixed",Activities!E32,IF(Activities!D32="Triangular",(Activities!F32+Activities!G32+Activities!H32)/3,IF(Activities!D32="Beta-PERT",(Activities!F32+4*Activities!G32+Activities!H32)/6,IF(Activities!D32="Normal",Activities!I32,IF(Activities!D32="Uniform",(Activities!F32+Activities!H32)/2,IF(OR(Activities!D32="Exponential",Activities!D32="Lognormal",Activities!D32="Gamma"),Activities!I32,NA()))))))</f>
         <v>2.1666666666666665</v>
       </c>
       <c r="D32" s="50">
@@ -7393,7 +7492,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:M99"/>
+  <dimension ref="A1:T99"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="11.625" style="9" customWidth="1"/>
@@ -7405,7 +7504,14 @@
     <col min="8" max="11" width="14" style="9" customWidth="1"/>
     <col min="12" max="12" width="13" style="9" customWidth="1"/>
     <col min="13" max="13" width="15.75" style="9" customWidth="1"/>
-    <col min="14" max="16384" width="9" style="2"/>
+    <col min="14" max="14" width="24" customWidth="1"/>
+    <col min="15" max="15" width="24" customWidth="1"/>
+    <col min="16" max="16" width="24" customWidth="1"/>
+    <col min="17" max="17" width="24" customWidth="1"/>
+    <col min="18" max="18" width="24" customWidth="1"/>
+    <col min="19" max="19" width="24" customWidth="1"/>
+    <col min="20" max="20" width="24" customWidth="1"/>
+    <col min="21" max="16384" width="9" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13" s="1" customFormat="1" ht="26.25" customHeight="1">
@@ -7425,7 +7531,7 @@
       <c r="L1" s="25"/>
       <c r="M1" s="25"/>
     </row>
-    <row r="2" spans="1:13" ht="30" customHeight="1">
+    <row r="2" spans="1:13" ht="65" customHeight="1">
       <c r="A2" s="15" t="s">
         <v>133</v>
       </c>
@@ -7464,6 +7570,41 @@
       </c>
       <c r="M2" s="15" t="s">
         <v>145</v>
+      </c>
+      <c r="N2" s="63" t="inlineStr">
+        <is>
+          <t>Cost_Model</t>
+        </is>
+      </c>
+      <c r="O2" s="64" t="inlineStr">
+        <is>
+          <t>Cost_Fixed</t>
+        </is>
+      </c>
+      <c r="P2" s="65" t="inlineStr">
+        <is>
+          <t>Cost_Min</t>
+        </is>
+      </c>
+      <c r="Q2" s="66" t="inlineStr">
+        <is>
+          <t>Cost_MostLikely</t>
+        </is>
+      </c>
+      <c r="R2" s="67" t="inlineStr">
+        <is>
+          <t>Cost_Max</t>
+        </is>
+      </c>
+      <c r="S2" s="68" t="inlineStr">
+        <is>
+          <t>Cost_Mean</t>
+        </is>
+      </c>
+      <c r="T2" s="69" t="inlineStr">
+        <is>
+          <t>Cost_SD</t>
+        </is>
       </c>
     </row>
     <row r="3" spans="1:13" ht="15" customHeight="1">
@@ -7496,6 +7637,13 @@
       <c r="M3" s="27" t="s">
         <v>149</v>
       </c>
+      <c r="N3" s="6"/>
+      <c r="O3" s="21"/>
+      <c r="P3" s="21"/>
+      <c r="Q3" s="21"/>
+      <c r="R3" s="21"/>
+      <c r="S3" s="21"/>
+      <c r="T3" s="21"/>
     </row>
     <row r="4" spans="1:13" ht="15" customHeight="1">
       <c r="A4" s="19" t="s">
@@ -7533,6 +7681,13 @@
       <c r="M4" s="27" t="s">
         <v>149</v>
       </c>
+      <c r="N4" s="6"/>
+      <c r="O4" s="21"/>
+      <c r="P4" s="21"/>
+      <c r="Q4" s="21"/>
+      <c r="R4" s="21"/>
+      <c r="S4" s="21"/>
+      <c r="T4" s="21"/>
     </row>
     <row r="5" spans="1:13" ht="15" customHeight="1">
       <c r="A5" s="19" t="s">
@@ -7570,6 +7725,13 @@
       <c r="M5" s="27" t="s">
         <v>149</v>
       </c>
+      <c r="N5" s="6"/>
+      <c r="O5" s="21"/>
+      <c r="P5" s="21"/>
+      <c r="Q5" s="21"/>
+      <c r="R5" s="21"/>
+      <c r="S5" s="21"/>
+      <c r="T5" s="21"/>
     </row>
     <row r="6" spans="1:13" ht="15" customHeight="1">
       <c r="A6" s="19" t="s">
@@ -7605,6 +7767,13 @@
       <c r="M6" s="27" t="s">
         <v>149</v>
       </c>
+      <c r="N6" s="6"/>
+      <c r="O6" s="21"/>
+      <c r="P6" s="21"/>
+      <c r="Q6" s="21"/>
+      <c r="R6" s="21"/>
+      <c r="S6" s="21"/>
+      <c r="T6" s="21"/>
     </row>
     <row r="7" spans="1:13" ht="15" customHeight="1">
       <c r="A7" s="19" t="s">
@@ -7638,6 +7807,13 @@
       <c r="M7" s="27" t="s">
         <v>149</v>
       </c>
+      <c r="N7" s="6"/>
+      <c r="O7" s="21"/>
+      <c r="P7" s="21"/>
+      <c r="Q7" s="21"/>
+      <c r="R7" s="21"/>
+      <c r="S7" s="21"/>
+      <c r="T7" s="21"/>
     </row>
     <row r="8" spans="1:13" ht="15" customHeight="1">
       <c r="A8" s="19" t="s">
@@ -7675,6 +7851,13 @@
       <c r="M8" s="27" t="s">
         <v>149</v>
       </c>
+      <c r="N8" s="6"/>
+      <c r="O8" s="21"/>
+      <c r="P8" s="21"/>
+      <c r="Q8" s="21"/>
+      <c r="R8" s="21"/>
+      <c r="S8" s="21"/>
+      <c r="T8" s="21"/>
     </row>
     <row r="9" spans="1:13" ht="15" customHeight="1">
       <c r="A9" s="19" t="s">
@@ -7712,6 +7895,13 @@
       <c r="M9" s="27" t="s">
         <v>149</v>
       </c>
+      <c r="N9" s="6"/>
+      <c r="O9" s="21"/>
+      <c r="P9" s="21"/>
+      <c r="Q9" s="21"/>
+      <c r="R9" s="21"/>
+      <c r="S9" s="21"/>
+      <c r="T9" s="21"/>
     </row>
     <row r="10" spans="1:13" ht="15" customHeight="1">
       <c r="A10" s="19" t="s">
@@ -7747,6 +7937,13 @@
       <c r="M10" s="27" t="s">
         <v>149</v>
       </c>
+      <c r="N10" s="6"/>
+      <c r="O10" s="21"/>
+      <c r="P10" s="21"/>
+      <c r="Q10" s="21"/>
+      <c r="R10" s="21"/>
+      <c r="S10" s="21"/>
+      <c r="T10" s="21"/>
     </row>
     <row r="11" spans="1:13" ht="15" customHeight="1">
       <c r="A11" s="19" t="s">
@@ -7780,6 +7977,13 @@
       <c r="M11" s="27" t="s">
         <v>149</v>
       </c>
+      <c r="N11" s="6"/>
+      <c r="O11" s="21"/>
+      <c r="P11" s="21"/>
+      <c r="Q11" s="21"/>
+      <c r="R11" s="21"/>
+      <c r="S11" s="21"/>
+      <c r="T11" s="21"/>
     </row>
     <row r="12" spans="1:13" ht="15" customHeight="1">
       <c r="A12" s="19" t="s">
@@ -7817,6 +8021,13 @@
       <c r="M12" s="27" t="s">
         <v>149</v>
       </c>
+      <c r="N12" s="6"/>
+      <c r="O12" s="21"/>
+      <c r="P12" s="21"/>
+      <c r="Q12" s="21"/>
+      <c r="R12" s="21"/>
+      <c r="S12" s="21"/>
+      <c r="T12" s="21"/>
     </row>
     <row r="13" spans="1:13" ht="15" customHeight="1">
       <c r="A13" s="19" t="s">
@@ -7854,6 +8065,13 @@
       <c r="M13" s="27" t="s">
         <v>149</v>
       </c>
+      <c r="N13" s="6"/>
+      <c r="O13" s="21"/>
+      <c r="P13" s="21"/>
+      <c r="Q13" s="21"/>
+      <c r="R13" s="21"/>
+      <c r="S13" s="21"/>
+      <c r="T13" s="21"/>
     </row>
     <row r="14" spans="1:13" ht="15" customHeight="1">
       <c r="A14" s="19" t="s">
@@ -7889,6 +8107,13 @@
       <c r="M14" s="27" t="s">
         <v>149</v>
       </c>
+      <c r="N14" s="6"/>
+      <c r="O14" s="21"/>
+      <c r="P14" s="21"/>
+      <c r="Q14" s="21"/>
+      <c r="R14" s="21"/>
+      <c r="S14" s="21"/>
+      <c r="T14" s="21"/>
     </row>
     <row r="15" spans="1:13" ht="15" customHeight="1">
       <c r="A15" s="19" t="s">
@@ -7922,6 +8147,13 @@
       <c r="M15" s="27" t="s">
         <v>149</v>
       </c>
+      <c r="N15" s="6"/>
+      <c r="O15" s="21"/>
+      <c r="P15" s="21"/>
+      <c r="Q15" s="21"/>
+      <c r="R15" s="21"/>
+      <c r="S15" s="21"/>
+      <c r="T15" s="21"/>
     </row>
     <row r="16" spans="1:13" ht="15" customHeight="1">
       <c r="A16" s="19" t="s">
@@ -7959,6 +8191,13 @@
       <c r="M16" s="27" t="s">
         <v>149</v>
       </c>
+      <c r="N16" s="6"/>
+      <c r="O16" s="21"/>
+      <c r="P16" s="21"/>
+      <c r="Q16" s="21"/>
+      <c r="R16" s="21"/>
+      <c r="S16" s="21"/>
+      <c r="T16" s="21"/>
     </row>
     <row r="17" spans="1:13" ht="15" customHeight="1">
       <c r="A17" s="19" t="s">
@@ -7996,6 +8235,13 @@
       <c r="M17" s="27" t="s">
         <v>71</v>
       </c>
+      <c r="N17" s="6"/>
+      <c r="O17" s="21"/>
+      <c r="P17" s="21"/>
+      <c r="Q17" s="21"/>
+      <c r="R17" s="21"/>
+      <c r="S17" s="21"/>
+      <c r="T17" s="21"/>
     </row>
     <row r="18" spans="1:13" ht="15" customHeight="1">
       <c r="A18" s="19" t="s">
@@ -8031,6 +8277,13 @@
       <c r="M18" s="27" t="s">
         <v>149</v>
       </c>
+      <c r="N18" s="6"/>
+      <c r="O18" s="21"/>
+      <c r="P18" s="21"/>
+      <c r="Q18" s="21"/>
+      <c r="R18" s="21"/>
+      <c r="S18" s="21"/>
+      <c r="T18" s="21"/>
     </row>
     <row r="19" spans="1:13" ht="15" customHeight="1">
       <c r="A19" s="19" t="s">
@@ -8064,6 +8317,13 @@
       <c r="M19" s="27" t="s">
         <v>149</v>
       </c>
+      <c r="N19" s="6"/>
+      <c r="O19" s="21"/>
+      <c r="P19" s="21"/>
+      <c r="Q19" s="21"/>
+      <c r="R19" s="21"/>
+      <c r="S19" s="21"/>
+      <c r="T19" s="21"/>
     </row>
     <row r="20" spans="1:13" ht="15" customHeight="1">
       <c r="A20" s="19" t="s">
@@ -8101,6 +8361,13 @@
       <c r="M20" s="27" t="s">
         <v>149</v>
       </c>
+      <c r="N20" s="6"/>
+      <c r="O20" s="21"/>
+      <c r="P20" s="21"/>
+      <c r="Q20" s="21"/>
+      <c r="R20" s="21"/>
+      <c r="S20" s="21"/>
+      <c r="T20" s="21"/>
     </row>
     <row r="21" spans="1:13" ht="15" customHeight="1">
       <c r="A21" s="19" t="s">
@@ -8138,6 +8405,13 @@
       <c r="M21" s="27" t="s">
         <v>149</v>
       </c>
+      <c r="N21" s="6"/>
+      <c r="O21" s="21"/>
+      <c r="P21" s="21"/>
+      <c r="Q21" s="21"/>
+      <c r="R21" s="21"/>
+      <c r="S21" s="21"/>
+      <c r="T21" s="21"/>
     </row>
     <row r="22" spans="1:13" ht="15" customHeight="1">
       <c r="A22" s="19" t="s">
@@ -8173,6 +8447,13 @@
       <c r="M22" s="27" t="s">
         <v>149</v>
       </c>
+      <c r="N22" s="6"/>
+      <c r="O22" s="21"/>
+      <c r="P22" s="21"/>
+      <c r="Q22" s="21"/>
+      <c r="R22" s="21"/>
+      <c r="S22" s="21"/>
+      <c r="T22" s="21"/>
     </row>
     <row r="23" spans="1:13" ht="15" customHeight="1">
       <c r="A23" s="19" t="s">
@@ -8206,6 +8487,13 @@
       <c r="M23" s="27" t="s">
         <v>149</v>
       </c>
+      <c r="N23" s="6"/>
+      <c r="O23" s="21"/>
+      <c r="P23" s="21"/>
+      <c r="Q23" s="21"/>
+      <c r="R23" s="21"/>
+      <c r="S23" s="21"/>
+      <c r="T23" s="21"/>
     </row>
     <row r="24" spans="1:13" ht="15" customHeight="1">
       <c r="A24" s="19" t="s">
@@ -8243,6 +8531,13 @@
       <c r="M24" s="27" t="s">
         <v>71</v>
       </c>
+      <c r="N24" s="6"/>
+      <c r="O24" s="21"/>
+      <c r="P24" s="21"/>
+      <c r="Q24" s="21"/>
+      <c r="R24" s="21"/>
+      <c r="S24" s="21"/>
+      <c r="T24" s="21"/>
     </row>
     <row r="25" spans="1:13" ht="15" customHeight="1">
       <c r="A25" s="19" t="s">
@@ -8280,6 +8575,13 @@
       <c r="M25" s="27" t="s">
         <v>71</v>
       </c>
+      <c r="N25" s="6"/>
+      <c r="O25" s="21"/>
+      <c r="P25" s="21"/>
+      <c r="Q25" s="21"/>
+      <c r="R25" s="21"/>
+      <c r="S25" s="21"/>
+      <c r="T25" s="21"/>
     </row>
     <row r="26" spans="1:13" ht="15" customHeight="1">
       <c r="A26" s="19" t="s">
@@ -8315,6 +8617,13 @@
       <c r="M26" s="27" t="s">
         <v>71</v>
       </c>
+      <c r="N26" s="6"/>
+      <c r="O26" s="21"/>
+      <c r="P26" s="21"/>
+      <c r="Q26" s="21"/>
+      <c r="R26" s="21"/>
+      <c r="S26" s="21"/>
+      <c r="T26" s="21"/>
     </row>
     <row r="27" spans="1:13" ht="15" customHeight="1">
       <c r="A27" s="19" t="s">
@@ -8348,6 +8657,13 @@
       <c r="M27" s="27" t="s">
         <v>149</v>
       </c>
+      <c r="N27" s="6"/>
+      <c r="O27" s="21"/>
+      <c r="P27" s="21"/>
+      <c r="Q27" s="21"/>
+      <c r="R27" s="21"/>
+      <c r="S27" s="21"/>
+      <c r="T27" s="21"/>
     </row>
     <row r="28" spans="1:13" ht="15" customHeight="1">
       <c r="A28" s="19" t="s">
@@ -8385,6 +8701,13 @@
       <c r="M28" s="27" t="s">
         <v>149</v>
       </c>
+      <c r="N28" s="6"/>
+      <c r="O28" s="21"/>
+      <c r="P28" s="21"/>
+      <c r="Q28" s="21"/>
+      <c r="R28" s="21"/>
+      <c r="S28" s="21"/>
+      <c r="T28" s="21"/>
     </row>
     <row r="29" spans="1:13" ht="15" customHeight="1">
       <c r="A29" s="19" t="s">
@@ -8422,6 +8745,13 @@
       <c r="M29" s="27" t="s">
         <v>149</v>
       </c>
+      <c r="N29" s="6"/>
+      <c r="O29" s="21"/>
+      <c r="P29" s="21"/>
+      <c r="Q29" s="21"/>
+      <c r="R29" s="21"/>
+      <c r="S29" s="21"/>
+      <c r="T29" s="21"/>
     </row>
     <row r="30" spans="1:13" ht="15" customHeight="1">
       <c r="A30" s="19" t="s">
@@ -8457,6 +8787,13 @@
       <c r="M30" s="27" t="s">
         <v>149</v>
       </c>
+      <c r="N30" s="6"/>
+      <c r="O30" s="21"/>
+      <c r="P30" s="21"/>
+      <c r="Q30" s="21"/>
+      <c r="R30" s="21"/>
+      <c r="S30" s="21"/>
+      <c r="T30" s="21"/>
     </row>
     <row r="31" spans="1:13" ht="15" customHeight="1">
       <c r="A31" s="19" t="s">
@@ -8494,6 +8831,13 @@
       <c r="M31" s="27" t="s">
         <v>71</v>
       </c>
+      <c r="N31" s="6"/>
+      <c r="O31" s="21"/>
+      <c r="P31" s="21"/>
+      <c r="Q31" s="21"/>
+      <c r="R31" s="21"/>
+      <c r="S31" s="21"/>
+      <c r="T31" s="21"/>
     </row>
     <row r="32" spans="1:13" ht="15" customHeight="1">
       <c r="A32" s="19" t="s">
@@ -8531,6 +8875,13 @@
       <c r="M32" s="27" t="s">
         <v>71</v>
       </c>
+      <c r="N32" s="6"/>
+      <c r="O32" s="21"/>
+      <c r="P32" s="21"/>
+      <c r="Q32" s="21"/>
+      <c r="R32" s="21"/>
+      <c r="S32" s="21"/>
+      <c r="T32" s="21"/>
     </row>
     <row r="33" spans="1:13">
       <c r="A33" s="19"/>
@@ -8546,6 +8897,13 @@
       <c r="K33" s="23"/>
       <c r="L33" s="27"/>
       <c r="M33" s="27"/>
+      <c r="N33" s="6"/>
+      <c r="O33" s="21"/>
+      <c r="P33" s="21"/>
+      <c r="Q33" s="21"/>
+      <c r="R33" s="21"/>
+      <c r="S33" s="21"/>
+      <c r="T33" s="21"/>
     </row>
     <row r="34" spans="1:13">
       <c r="A34" s="19"/>
@@ -8561,6 +8919,13 @@
       <c r="K34" s="23"/>
       <c r="L34" s="27"/>
       <c r="M34" s="27"/>
+      <c r="N34" s="6"/>
+      <c r="O34" s="21"/>
+      <c r="P34" s="21"/>
+      <c r="Q34" s="21"/>
+      <c r="R34" s="21"/>
+      <c r="S34" s="21"/>
+      <c r="T34" s="21"/>
     </row>
     <row r="35" spans="1:13" s="1" customFormat="1">
       <c r="A35" s="20"/>
@@ -8576,6 +8941,13 @@
       <c r="K35" s="24"/>
       <c r="L35" s="27"/>
       <c r="M35" s="27"/>
+      <c r="N35" s="18"/>
+      <c r="O35" s="20"/>
+      <c r="P35" s="20"/>
+      <c r="Q35" s="20"/>
+      <c r="R35" s="20"/>
+      <c r="S35" s="20"/>
+      <c r="T35" s="20"/>
     </row>
     <row r="36" spans="1:13" s="1" customFormat="1">
       <c r="A36" s="20"/>
@@ -8591,6 +8963,13 @@
       <c r="K36" s="24"/>
       <c r="L36" s="27"/>
       <c r="M36" s="27"/>
+      <c r="N36" s="18"/>
+      <c r="O36" s="20"/>
+      <c r="P36" s="20"/>
+      <c r="Q36" s="20"/>
+      <c r="R36" s="20"/>
+      <c r="S36" s="20"/>
+      <c r="T36" s="20"/>
     </row>
     <row r="37" spans="1:13" s="1" customFormat="1">
       <c r="A37" s="20"/>
@@ -8606,6 +8985,13 @@
       <c r="K37" s="24"/>
       <c r="L37" s="27"/>
       <c r="M37" s="27"/>
+      <c r="N37" s="18"/>
+      <c r="O37" s="20"/>
+      <c r="P37" s="20"/>
+      <c r="Q37" s="20"/>
+      <c r="R37" s="20"/>
+      <c r="S37" s="20"/>
+      <c r="T37" s="20"/>
     </row>
     <row r="38" spans="1:13" s="1" customFormat="1">
       <c r="A38" s="20"/>
@@ -8621,6 +9007,13 @@
       <c r="K38" s="24"/>
       <c r="L38" s="27"/>
       <c r="M38" s="27"/>
+      <c r="N38" s="18"/>
+      <c r="O38" s="20"/>
+      <c r="P38" s="20"/>
+      <c r="Q38" s="20"/>
+      <c r="R38" s="20"/>
+      <c r="S38" s="20"/>
+      <c r="T38" s="20"/>
     </row>
     <row r="39" spans="1:13" s="1" customFormat="1">
       <c r="A39" s="20"/>
@@ -8636,6 +9029,13 @@
       <c r="K39" s="24"/>
       <c r="L39" s="27"/>
       <c r="M39" s="27"/>
+      <c r="N39" s="18"/>
+      <c r="O39" s="20"/>
+      <c r="P39" s="20"/>
+      <c r="Q39" s="20"/>
+      <c r="R39" s="20"/>
+      <c r="S39" s="20"/>
+      <c r="T39" s="20"/>
     </row>
     <row r="40" spans="1:13" s="1" customFormat="1">
       <c r="A40" s="20"/>
@@ -8651,6 +9051,13 @@
       <c r="K40" s="24"/>
       <c r="L40" s="27"/>
       <c r="M40" s="27"/>
+      <c r="N40" s="18"/>
+      <c r="O40" s="20"/>
+      <c r="P40" s="20"/>
+      <c r="Q40" s="20"/>
+      <c r="R40" s="20"/>
+      <c r="S40" s="20"/>
+      <c r="T40" s="20"/>
     </row>
     <row r="41" spans="1:13" s="1" customFormat="1">
       <c r="A41" s="20"/>
@@ -8666,6 +9073,13 @@
       <c r="K41" s="24"/>
       <c r="L41" s="27"/>
       <c r="M41" s="27"/>
+      <c r="N41" s="18"/>
+      <c r="O41" s="20"/>
+      <c r="P41" s="20"/>
+      <c r="Q41" s="20"/>
+      <c r="R41" s="20"/>
+      <c r="S41" s="20"/>
+      <c r="T41" s="20"/>
     </row>
     <row r="42" spans="1:13" s="1" customFormat="1">
       <c r="A42" s="20"/>
@@ -8681,6 +9095,13 @@
       <c r="K42" s="24"/>
       <c r="L42" s="27"/>
       <c r="M42" s="27"/>
+      <c r="N42" s="18"/>
+      <c r="O42" s="20"/>
+      <c r="P42" s="20"/>
+      <c r="Q42" s="20"/>
+      <c r="R42" s="20"/>
+      <c r="S42" s="20"/>
+      <c r="T42" s="20"/>
     </row>
     <row r="43" spans="1:13" s="1" customFormat="1">
       <c r="A43" s="20"/>
@@ -8696,6 +9117,13 @@
       <c r="K43" s="24"/>
       <c r="L43" s="27"/>
       <c r="M43" s="27"/>
+      <c r="N43" s="18"/>
+      <c r="O43" s="20"/>
+      <c r="P43" s="20"/>
+      <c r="Q43" s="20"/>
+      <c r="R43" s="20"/>
+      <c r="S43" s="20"/>
+      <c r="T43" s="20"/>
     </row>
     <row r="44" spans="1:13" s="1" customFormat="1">
       <c r="A44" s="20"/>
@@ -8711,6 +9139,13 @@
       <c r="K44" s="24"/>
       <c r="L44" s="27"/>
       <c r="M44" s="27"/>
+      <c r="N44" s="18"/>
+      <c r="O44" s="20"/>
+      <c r="P44" s="20"/>
+      <c r="Q44" s="20"/>
+      <c r="R44" s="20"/>
+      <c r="S44" s="20"/>
+      <c r="T44" s="20"/>
     </row>
     <row r="45" spans="1:13" s="1" customFormat="1">
       <c r="A45" s="20"/>
@@ -8726,6 +9161,13 @@
       <c r="K45" s="24"/>
       <c r="L45" s="27"/>
       <c r="M45" s="27"/>
+      <c r="N45" s="18"/>
+      <c r="O45" s="20"/>
+      <c r="P45" s="20"/>
+      <c r="Q45" s="20"/>
+      <c r="R45" s="20"/>
+      <c r="S45" s="20"/>
+      <c r="T45" s="20"/>
     </row>
     <row r="46" spans="1:13" s="1" customFormat="1">
       <c r="A46" s="20"/>
@@ -8741,6 +9183,13 @@
       <c r="K46" s="24"/>
       <c r="L46" s="27"/>
       <c r="M46" s="27"/>
+      <c r="N46" s="18"/>
+      <c r="O46" s="20"/>
+      <c r="P46" s="20"/>
+      <c r="Q46" s="20"/>
+      <c r="R46" s="20"/>
+      <c r="S46" s="20"/>
+      <c r="T46" s="20"/>
     </row>
     <row r="47" spans="1:13" s="1" customFormat="1">
       <c r="A47" s="20"/>
@@ -8756,6 +9205,13 @@
       <c r="K47" s="24"/>
       <c r="L47" s="27"/>
       <c r="M47" s="27"/>
+      <c r="N47" s="18"/>
+      <c r="O47" s="20"/>
+      <c r="P47" s="20"/>
+      <c r="Q47" s="20"/>
+      <c r="R47" s="20"/>
+      <c r="S47" s="20"/>
+      <c r="T47" s="20"/>
     </row>
     <row r="48" spans="1:13" s="1" customFormat="1">
       <c r="A48" s="20"/>
@@ -8771,6 +9227,13 @@
       <c r="K48" s="24"/>
       <c r="L48" s="27"/>
       <c r="M48" s="27"/>
+      <c r="N48" s="18"/>
+      <c r="O48" s="20"/>
+      <c r="P48" s="20"/>
+      <c r="Q48" s="20"/>
+      <c r="R48" s="20"/>
+      <c r="S48" s="20"/>
+      <c r="T48" s="20"/>
     </row>
     <row r="49" spans="1:13" s="1" customFormat="1">
       <c r="A49" s="20"/>
@@ -8786,6 +9249,13 @@
       <c r="K49" s="24"/>
       <c r="L49" s="27"/>
       <c r="M49" s="27"/>
+      <c r="N49" s="18"/>
+      <c r="O49" s="20"/>
+      <c r="P49" s="20"/>
+      <c r="Q49" s="20"/>
+      <c r="R49" s="20"/>
+      <c r="S49" s="20"/>
+      <c r="T49" s="20"/>
     </row>
     <row r="50" spans="1:13" s="1" customFormat="1">
       <c r="A50" s="20"/>
@@ -8801,6 +9271,13 @@
       <c r="K50" s="24"/>
       <c r="L50" s="27"/>
       <c r="M50" s="27"/>
+      <c r="N50" s="18"/>
+      <c r="O50" s="20"/>
+      <c r="P50" s="20"/>
+      <c r="Q50" s="20"/>
+      <c r="R50" s="20"/>
+      <c r="S50" s="20"/>
+      <c r="T50" s="20"/>
     </row>
     <row r="51" spans="1:13" s="1" customFormat="1">
       <c r="A51" s="20"/>
@@ -8816,6 +9293,13 @@
       <c r="K51" s="24"/>
       <c r="L51" s="27"/>
       <c r="M51" s="27"/>
+      <c r="N51" s="18"/>
+      <c r="O51" s="20"/>
+      <c r="P51" s="20"/>
+      <c r="Q51" s="20"/>
+      <c r="R51" s="20"/>
+      <c r="S51" s="20"/>
+      <c r="T51" s="20"/>
     </row>
     <row r="52" spans="1:13" s="1" customFormat="1">
       <c r="A52" s="20"/>
@@ -8831,6 +9315,13 @@
       <c r="K52" s="24"/>
       <c r="L52" s="27"/>
       <c r="M52" s="27"/>
+      <c r="N52" s="18"/>
+      <c r="O52" s="20"/>
+      <c r="P52" s="20"/>
+      <c r="Q52" s="20"/>
+      <c r="R52" s="20"/>
+      <c r="S52" s="20"/>
+      <c r="T52" s="20"/>
     </row>
     <row r="53" spans="1:13" s="1" customFormat="1">
       <c r="A53" s="20"/>
@@ -8846,6 +9337,13 @@
       <c r="K53" s="24"/>
       <c r="L53" s="27"/>
       <c r="M53" s="27"/>
+      <c r="N53" s="18"/>
+      <c r="O53" s="20"/>
+      <c r="P53" s="20"/>
+      <c r="Q53" s="20"/>
+      <c r="R53" s="20"/>
+      <c r="S53" s="20"/>
+      <c r="T53" s="20"/>
     </row>
     <row r="54" spans="1:13" s="1" customFormat="1">
       <c r="A54" s="20"/>
@@ -8861,6 +9359,13 @@
       <c r="K54" s="24"/>
       <c r="L54" s="27"/>
       <c r="M54" s="27"/>
+      <c r="N54" s="18"/>
+      <c r="O54" s="20"/>
+      <c r="P54" s="20"/>
+      <c r="Q54" s="20"/>
+      <c r="R54" s="20"/>
+      <c r="S54" s="20"/>
+      <c r="T54" s="20"/>
     </row>
     <row r="55" spans="1:13" s="1" customFormat="1">
       <c r="A55" s="20"/>
@@ -8876,6 +9381,13 @@
       <c r="K55" s="24"/>
       <c r="L55" s="27"/>
       <c r="M55" s="27"/>
+      <c r="N55" s="18"/>
+      <c r="O55" s="20"/>
+      <c r="P55" s="20"/>
+      <c r="Q55" s="20"/>
+      <c r="R55" s="20"/>
+      <c r="S55" s="20"/>
+      <c r="T55" s="20"/>
     </row>
     <row r="56" spans="1:13" s="1" customFormat="1">
       <c r="A56" s="20"/>
@@ -8891,6 +9403,13 @@
       <c r="K56" s="24"/>
       <c r="L56" s="27"/>
       <c r="M56" s="27"/>
+      <c r="N56" s="18"/>
+      <c r="O56" s="20"/>
+      <c r="P56" s="20"/>
+      <c r="Q56" s="20"/>
+      <c r="R56" s="20"/>
+      <c r="S56" s="20"/>
+      <c r="T56" s="20"/>
     </row>
     <row r="57" spans="1:13" s="1" customFormat="1">
       <c r="A57" s="20"/>
@@ -8906,6 +9425,13 @@
       <c r="K57" s="24"/>
       <c r="L57" s="27"/>
       <c r="M57" s="27"/>
+      <c r="N57" s="18"/>
+      <c r="O57" s="20"/>
+      <c r="P57" s="20"/>
+      <c r="Q57" s="20"/>
+      <c r="R57" s="20"/>
+      <c r="S57" s="20"/>
+      <c r="T57" s="20"/>
     </row>
     <row r="58" spans="1:13" s="1" customFormat="1">
       <c r="A58" s="20"/>
@@ -8921,6 +9447,13 @@
       <c r="K58" s="24"/>
       <c r="L58" s="27"/>
       <c r="M58" s="27"/>
+      <c r="N58" s="18"/>
+      <c r="O58" s="20"/>
+      <c r="P58" s="20"/>
+      <c r="Q58" s="20"/>
+      <c r="R58" s="20"/>
+      <c r="S58" s="20"/>
+      <c r="T58" s="20"/>
     </row>
     <row r="59" spans="1:13" s="1" customFormat="1">
       <c r="A59" s="20"/>
@@ -8936,6 +9469,13 @@
       <c r="K59" s="24"/>
       <c r="L59" s="27"/>
       <c r="M59" s="27"/>
+      <c r="N59" s="18"/>
+      <c r="O59" s="20"/>
+      <c r="P59" s="20"/>
+      <c r="Q59" s="20"/>
+      <c r="R59" s="20"/>
+      <c r="S59" s="20"/>
+      <c r="T59" s="20"/>
     </row>
     <row r="60" spans="1:13" s="1" customFormat="1">
       <c r="A60" s="20"/>
@@ -8951,6 +9491,13 @@
       <c r="K60" s="24"/>
       <c r="L60" s="27"/>
       <c r="M60" s="27"/>
+      <c r="N60" s="18"/>
+      <c r="O60" s="20"/>
+      <c r="P60" s="20"/>
+      <c r="Q60" s="20"/>
+      <c r="R60" s="20"/>
+      <c r="S60" s="20"/>
+      <c r="T60" s="20"/>
     </row>
     <row r="61" spans="1:13" s="1" customFormat="1">
       <c r="A61" s="20"/>
@@ -8966,6 +9513,13 @@
       <c r="K61" s="24"/>
       <c r="L61" s="27"/>
       <c r="M61" s="27"/>
+      <c r="N61" s="18"/>
+      <c r="O61" s="20"/>
+      <c r="P61" s="20"/>
+      <c r="Q61" s="20"/>
+      <c r="R61" s="20"/>
+      <c r="S61" s="20"/>
+      <c r="T61" s="20"/>
     </row>
     <row r="62" spans="1:13" s="1" customFormat="1">
       <c r="A62" s="20"/>
@@ -8981,6 +9535,13 @@
       <c r="K62" s="24"/>
       <c r="L62" s="27"/>
       <c r="M62" s="27"/>
+      <c r="N62" s="18"/>
+      <c r="O62" s="20"/>
+      <c r="P62" s="20"/>
+      <c r="Q62" s="20"/>
+      <c r="R62" s="20"/>
+      <c r="S62" s="20"/>
+      <c r="T62" s="20"/>
     </row>
     <row r="63" spans="1:13" s="1" customFormat="1">
       <c r="A63" s="20"/>
@@ -8996,6 +9557,13 @@
       <c r="K63" s="24"/>
       <c r="L63" s="27"/>
       <c r="M63" s="27"/>
+      <c r="N63" s="18"/>
+      <c r="O63" s="20"/>
+      <c r="P63" s="20"/>
+      <c r="Q63" s="20"/>
+      <c r="R63" s="20"/>
+      <c r="S63" s="20"/>
+      <c r="T63" s="20"/>
     </row>
     <row r="64" spans="1:13" s="1" customFormat="1">
       <c r="A64" s="20"/>
@@ -9011,6 +9579,13 @@
       <c r="K64" s="24"/>
       <c r="L64" s="27"/>
       <c r="M64" s="27"/>
+      <c r="N64" s="18"/>
+      <c r="O64" s="20"/>
+      <c r="P64" s="20"/>
+      <c r="Q64" s="20"/>
+      <c r="R64" s="20"/>
+      <c r="S64" s="20"/>
+      <c r="T64" s="20"/>
     </row>
     <row r="65" spans="1:13" s="1" customFormat="1">
       <c r="A65" s="20"/>
@@ -9026,6 +9601,13 @@
       <c r="K65" s="24"/>
       <c r="L65" s="27"/>
       <c r="M65" s="27"/>
+      <c r="N65" s="18"/>
+      <c r="O65" s="20"/>
+      <c r="P65" s="20"/>
+      <c r="Q65" s="20"/>
+      <c r="R65" s="20"/>
+      <c r="S65" s="20"/>
+      <c r="T65" s="20"/>
     </row>
     <row r="66" spans="1:13" s="1" customFormat="1">
       <c r="A66" s="20"/>
@@ -9041,6 +9623,13 @@
       <c r="K66" s="24"/>
       <c r="L66" s="27"/>
       <c r="M66" s="27"/>
+      <c r="N66" s="18"/>
+      <c r="O66" s="20"/>
+      <c r="P66" s="20"/>
+      <c r="Q66" s="20"/>
+      <c r="R66" s="20"/>
+      <c r="S66" s="20"/>
+      <c r="T66" s="20"/>
     </row>
     <row r="67" spans="1:13" s="1" customFormat="1">
       <c r="A67" s="20"/>
@@ -9056,6 +9645,13 @@
       <c r="K67" s="24"/>
       <c r="L67" s="27"/>
       <c r="M67" s="27"/>
+      <c r="N67" s="18"/>
+      <c r="O67" s="20"/>
+      <c r="P67" s="20"/>
+      <c r="Q67" s="20"/>
+      <c r="R67" s="20"/>
+      <c r="S67" s="20"/>
+      <c r="T67" s="20"/>
     </row>
     <row r="68" spans="1:13" s="1" customFormat="1">
       <c r="A68" s="20"/>
@@ -9071,6 +9667,13 @@
       <c r="K68" s="24"/>
       <c r="L68" s="27"/>
       <c r="M68" s="27"/>
+      <c r="N68" s="18"/>
+      <c r="O68" s="20"/>
+      <c r="P68" s="20"/>
+      <c r="Q68" s="20"/>
+      <c r="R68" s="20"/>
+      <c r="S68" s="20"/>
+      <c r="T68" s="20"/>
     </row>
     <row r="69" spans="1:13" s="1" customFormat="1">
       <c r="A69" s="20"/>
@@ -9086,6 +9689,13 @@
       <c r="K69" s="24"/>
       <c r="L69" s="27"/>
       <c r="M69" s="27"/>
+      <c r="N69" s="18"/>
+      <c r="O69" s="20"/>
+      <c r="P69" s="20"/>
+      <c r="Q69" s="20"/>
+      <c r="R69" s="20"/>
+      <c r="S69" s="20"/>
+      <c r="T69" s="20"/>
     </row>
     <row r="70" spans="1:13" s="1" customFormat="1">
       <c r="A70" s="20"/>
@@ -9101,6 +9711,13 @@
       <c r="K70" s="24"/>
       <c r="L70" s="27"/>
       <c r="M70" s="27"/>
+      <c r="N70" s="18"/>
+      <c r="O70" s="20"/>
+      <c r="P70" s="20"/>
+      <c r="Q70" s="20"/>
+      <c r="R70" s="20"/>
+      <c r="S70" s="20"/>
+      <c r="T70" s="20"/>
     </row>
     <row r="71" spans="1:13" s="1" customFormat="1">
       <c r="A71" s="20"/>
@@ -9116,6 +9733,13 @@
       <c r="K71" s="24"/>
       <c r="L71" s="27"/>
       <c r="M71" s="27"/>
+      <c r="N71" s="18"/>
+      <c r="O71" s="20"/>
+      <c r="P71" s="20"/>
+      <c r="Q71" s="20"/>
+      <c r="R71" s="20"/>
+      <c r="S71" s="20"/>
+      <c r="T71" s="20"/>
     </row>
     <row r="72" spans="1:13" s="1" customFormat="1">
       <c r="A72" s="20"/>
@@ -9131,6 +9755,13 @@
       <c r="K72" s="24"/>
       <c r="L72" s="27"/>
       <c r="M72" s="27"/>
+      <c r="N72" s="18"/>
+      <c r="O72" s="20"/>
+      <c r="P72" s="20"/>
+      <c r="Q72" s="20"/>
+      <c r="R72" s="20"/>
+      <c r="S72" s="20"/>
+      <c r="T72" s="20"/>
     </row>
     <row r="73" spans="1:13" s="1" customFormat="1">
       <c r="A73" s="20"/>
@@ -9146,6 +9777,13 @@
       <c r="K73" s="24"/>
       <c r="L73" s="27"/>
       <c r="M73" s="27"/>
+      <c r="N73" s="18"/>
+      <c r="O73" s="20"/>
+      <c r="P73" s="20"/>
+      <c r="Q73" s="20"/>
+      <c r="R73" s="20"/>
+      <c r="S73" s="20"/>
+      <c r="T73" s="20"/>
     </row>
     <row r="74" spans="1:13" s="1" customFormat="1">
       <c r="A74" s="20"/>
@@ -9161,6 +9799,13 @@
       <c r="K74" s="24"/>
       <c r="L74" s="27"/>
       <c r="M74" s="27"/>
+      <c r="N74" s="18"/>
+      <c r="O74" s="20"/>
+      <c r="P74" s="20"/>
+      <c r="Q74" s="20"/>
+      <c r="R74" s="20"/>
+      <c r="S74" s="20"/>
+      <c r="T74" s="20"/>
     </row>
     <row r="75" spans="1:13" s="1" customFormat="1">
       <c r="A75" s="20"/>
@@ -9176,6 +9821,13 @@
       <c r="K75" s="24"/>
       <c r="L75" s="27"/>
       <c r="M75" s="27"/>
+      <c r="N75" s="18"/>
+      <c r="O75" s="20"/>
+      <c r="P75" s="20"/>
+      <c r="Q75" s="20"/>
+      <c r="R75" s="20"/>
+      <c r="S75" s="20"/>
+      <c r="T75" s="20"/>
     </row>
     <row r="76" spans="1:13" s="1" customFormat="1">
       <c r="A76" s="20"/>
@@ -9191,6 +9843,13 @@
       <c r="K76" s="24"/>
       <c r="L76" s="27"/>
       <c r="M76" s="27"/>
+      <c r="N76" s="18"/>
+      <c r="O76" s="20"/>
+      <c r="P76" s="20"/>
+      <c r="Q76" s="20"/>
+      <c r="R76" s="20"/>
+      <c r="S76" s="20"/>
+      <c r="T76" s="20"/>
     </row>
     <row r="77" spans="1:13" s="1" customFormat="1">
       <c r="A77" s="20"/>
@@ -9206,6 +9865,13 @@
       <c r="K77" s="24"/>
       <c r="L77" s="27"/>
       <c r="M77" s="27"/>
+      <c r="N77" s="18"/>
+      <c r="O77" s="20"/>
+      <c r="P77" s="20"/>
+      <c r="Q77" s="20"/>
+      <c r="R77" s="20"/>
+      <c r="S77" s="20"/>
+      <c r="T77" s="20"/>
     </row>
     <row r="78" spans="1:13" s="1" customFormat="1">
       <c r="A78" s="20"/>
@@ -9221,6 +9887,13 @@
       <c r="K78" s="24"/>
       <c r="L78" s="27"/>
       <c r="M78" s="27"/>
+      <c r="N78" s="18"/>
+      <c r="O78" s="20"/>
+      <c r="P78" s="20"/>
+      <c r="Q78" s="20"/>
+      <c r="R78" s="20"/>
+      <c r="S78" s="20"/>
+      <c r="T78" s="20"/>
     </row>
     <row r="79" spans="1:13" s="1" customFormat="1">
       <c r="A79" s="20"/>
@@ -9236,6 +9909,13 @@
       <c r="K79" s="24"/>
       <c r="L79" s="27"/>
       <c r="M79" s="27"/>
+      <c r="N79" s="18"/>
+      <c r="O79" s="20"/>
+      <c r="P79" s="20"/>
+      <c r="Q79" s="20"/>
+      <c r="R79" s="20"/>
+      <c r="S79" s="20"/>
+      <c r="T79" s="20"/>
     </row>
     <row r="80" spans="1:13" s="1" customFormat="1">
       <c r="A80" s="20"/>
@@ -9251,6 +9931,13 @@
       <c r="K80" s="24"/>
       <c r="L80" s="27"/>
       <c r="M80" s="27"/>
+      <c r="N80" s="18"/>
+      <c r="O80" s="20"/>
+      <c r="P80" s="20"/>
+      <c r="Q80" s="20"/>
+      <c r="R80" s="20"/>
+      <c r="S80" s="20"/>
+      <c r="T80" s="20"/>
     </row>
     <row r="81" spans="1:13" s="1" customFormat="1">
       <c r="A81" s="20"/>
@@ -9266,6 +9953,13 @@
       <c r="K81" s="24"/>
       <c r="L81" s="27"/>
       <c r="M81" s="27"/>
+      <c r="N81" s="18"/>
+      <c r="O81" s="20"/>
+      <c r="P81" s="20"/>
+      <c r="Q81" s="20"/>
+      <c r="R81" s="20"/>
+      <c r="S81" s="20"/>
+      <c r="T81" s="20"/>
     </row>
     <row r="82" spans="1:13" s="1" customFormat="1">
       <c r="A82" s="20"/>
@@ -9281,6 +9975,13 @@
       <c r="K82" s="24"/>
       <c r="L82" s="27"/>
       <c r="M82" s="27"/>
+      <c r="N82" s="18"/>
+      <c r="O82" s="20"/>
+      <c r="P82" s="20"/>
+      <c r="Q82" s="20"/>
+      <c r="R82" s="20"/>
+      <c r="S82" s="20"/>
+      <c r="T82" s="20"/>
     </row>
     <row r="83" spans="1:13" s="1" customFormat="1">
       <c r="A83" s="20"/>
@@ -9296,6 +9997,13 @@
       <c r="K83" s="24"/>
       <c r="L83" s="27"/>
       <c r="M83" s="27"/>
+      <c r="N83" s="18"/>
+      <c r="O83" s="20"/>
+      <c r="P83" s="20"/>
+      <c r="Q83" s="20"/>
+      <c r="R83" s="20"/>
+      <c r="S83" s="20"/>
+      <c r="T83" s="20"/>
     </row>
     <row r="84" spans="1:13" s="1" customFormat="1">
       <c r="A84" s="20"/>
@@ -9311,6 +10019,13 @@
       <c r="K84" s="24"/>
       <c r="L84" s="27"/>
       <c r="M84" s="27"/>
+      <c r="N84" s="18"/>
+      <c r="O84" s="20"/>
+      <c r="P84" s="20"/>
+      <c r="Q84" s="20"/>
+      <c r="R84" s="20"/>
+      <c r="S84" s="20"/>
+      <c r="T84" s="20"/>
     </row>
     <row r="85" spans="1:13" s="1" customFormat="1">
       <c r="A85" s="20"/>
@@ -9326,6 +10041,13 @@
       <c r="K85" s="24"/>
       <c r="L85" s="27"/>
       <c r="M85" s="27"/>
+      <c r="N85" s="18"/>
+      <c r="O85" s="20"/>
+      <c r="P85" s="20"/>
+      <c r="Q85" s="20"/>
+      <c r="R85" s="20"/>
+      <c r="S85" s="20"/>
+      <c r="T85" s="20"/>
     </row>
     <row r="86" spans="1:13" s="1" customFormat="1">
       <c r="A86" s="20"/>
@@ -9341,6 +10063,13 @@
       <c r="K86" s="24"/>
       <c r="L86" s="27"/>
       <c r="M86" s="27"/>
+      <c r="N86" s="18"/>
+      <c r="O86" s="20"/>
+      <c r="P86" s="20"/>
+      <c r="Q86" s="20"/>
+      <c r="R86" s="20"/>
+      <c r="S86" s="20"/>
+      <c r="T86" s="20"/>
     </row>
     <row r="87" spans="1:13" s="1" customFormat="1">
       <c r="A87" s="20"/>
@@ -9356,6 +10085,13 @@
       <c r="K87" s="24"/>
       <c r="L87" s="27"/>
       <c r="M87" s="27"/>
+      <c r="N87" s="18"/>
+      <c r="O87" s="20"/>
+      <c r="P87" s="20"/>
+      <c r="Q87" s="20"/>
+      <c r="R87" s="20"/>
+      <c r="S87" s="20"/>
+      <c r="T87" s="20"/>
     </row>
     <row r="88" spans="1:13" s="1" customFormat="1">
       <c r="A88" s="20"/>
@@ -9371,6 +10107,13 @@
       <c r="K88" s="24"/>
       <c r="L88" s="27"/>
       <c r="M88" s="27"/>
+      <c r="N88" s="18"/>
+      <c r="O88" s="20"/>
+      <c r="P88" s="20"/>
+      <c r="Q88" s="20"/>
+      <c r="R88" s="20"/>
+      <c r="S88" s="20"/>
+      <c r="T88" s="20"/>
     </row>
     <row r="89" spans="1:13" s="1" customFormat="1">
       <c r="A89" s="20"/>
@@ -9386,6 +10129,13 @@
       <c r="K89" s="24"/>
       <c r="L89" s="27"/>
       <c r="M89" s="27"/>
+      <c r="N89" s="18"/>
+      <c r="O89" s="20"/>
+      <c r="P89" s="20"/>
+      <c r="Q89" s="20"/>
+      <c r="R89" s="20"/>
+      <c r="S89" s="20"/>
+      <c r="T89" s="20"/>
     </row>
     <row r="90" spans="1:13" s="1" customFormat="1">
       <c r="A90" s="20"/>
@@ -9401,6 +10151,13 @@
       <c r="K90" s="24"/>
       <c r="L90" s="27"/>
       <c r="M90" s="27"/>
+      <c r="N90" s="18"/>
+      <c r="O90" s="20"/>
+      <c r="P90" s="20"/>
+      <c r="Q90" s="20"/>
+      <c r="R90" s="20"/>
+      <c r="S90" s="20"/>
+      <c r="T90" s="20"/>
     </row>
     <row r="91" spans="1:13" s="1" customFormat="1">
       <c r="A91" s="20"/>
@@ -9416,6 +10173,13 @@
       <c r="K91" s="24"/>
       <c r="L91" s="27"/>
       <c r="M91" s="27"/>
+      <c r="N91" s="18"/>
+      <c r="O91" s="20"/>
+      <c r="P91" s="20"/>
+      <c r="Q91" s="20"/>
+      <c r="R91" s="20"/>
+      <c r="S91" s="20"/>
+      <c r="T91" s="20"/>
     </row>
     <row r="92" spans="1:13" s="1" customFormat="1">
       <c r="A92" s="20"/>
@@ -9431,6 +10195,13 @@
       <c r="K92" s="24"/>
       <c r="L92" s="27"/>
       <c r="M92" s="27"/>
+      <c r="N92" s="18"/>
+      <c r="O92" s="20"/>
+      <c r="P92" s="20"/>
+      <c r="Q92" s="20"/>
+      <c r="R92" s="20"/>
+      <c r="S92" s="20"/>
+      <c r="T92" s="20"/>
     </row>
     <row r="93" spans="1:13" s="1" customFormat="1">
       <c r="A93" s="20"/>
@@ -9446,6 +10217,13 @@
       <c r="K93" s="24"/>
       <c r="L93" s="27"/>
       <c r="M93" s="27"/>
+      <c r="N93" s="18"/>
+      <c r="O93" s="20"/>
+      <c r="P93" s="20"/>
+      <c r="Q93" s="20"/>
+      <c r="R93" s="20"/>
+      <c r="S93" s="20"/>
+      <c r="T93" s="20"/>
     </row>
     <row r="94" spans="1:13" s="1" customFormat="1">
       <c r="A94" s="20"/>
@@ -9461,6 +10239,13 @@
       <c r="K94" s="24"/>
       <c r="L94" s="27"/>
       <c r="M94" s="27"/>
+      <c r="N94" s="18"/>
+      <c r="O94" s="20"/>
+      <c r="P94" s="20"/>
+      <c r="Q94" s="20"/>
+      <c r="R94" s="20"/>
+      <c r="S94" s="20"/>
+      <c r="T94" s="20"/>
     </row>
     <row r="95" spans="1:13" s="1" customFormat="1">
       <c r="A95" s="20"/>
@@ -9476,6 +10261,13 @@
       <c r="K95" s="24"/>
       <c r="L95" s="27"/>
       <c r="M95" s="27"/>
+      <c r="N95" s="18"/>
+      <c r="O95" s="20"/>
+      <c r="P95" s="20"/>
+      <c r="Q95" s="20"/>
+      <c r="R95" s="20"/>
+      <c r="S95" s="20"/>
+      <c r="T95" s="20"/>
     </row>
     <row r="96" spans="1:13" s="1" customFormat="1">
       <c r="A96" s="20"/>
@@ -9491,6 +10283,13 @@
       <c r="K96" s="24"/>
       <c r="L96" s="27"/>
       <c r="M96" s="27"/>
+      <c r="N96" s="18"/>
+      <c r="O96" s="20"/>
+      <c r="P96" s="20"/>
+      <c r="Q96" s="20"/>
+      <c r="R96" s="20"/>
+      <c r="S96" s="20"/>
+      <c r="T96" s="20"/>
     </row>
     <row r="97" spans="1:13" s="1" customFormat="1">
       <c r="A97" s="20"/>
@@ -9506,6 +10305,13 @@
       <c r="K97" s="24"/>
       <c r="L97" s="27"/>
       <c r="M97" s="27"/>
+      <c r="N97" s="18"/>
+      <c r="O97" s="20"/>
+      <c r="P97" s="20"/>
+      <c r="Q97" s="20"/>
+      <c r="R97" s="20"/>
+      <c r="S97" s="20"/>
+      <c r="T97" s="20"/>
     </row>
     <row r="98" spans="1:13" s="1" customFormat="1">
       <c r="A98" s="20"/>
@@ -9521,6 +10327,13 @@
       <c r="K98" s="24"/>
       <c r="L98" s="27"/>
       <c r="M98" s="27"/>
+      <c r="N98" s="18"/>
+      <c r="O98" s="20"/>
+      <c r="P98" s="20"/>
+      <c r="Q98" s="20"/>
+      <c r="R98" s="20"/>
+      <c r="S98" s="20"/>
+      <c r="T98" s="20"/>
     </row>
     <row r="99" spans="1:13" s="1" customFormat="1">
       <c r="A99" s="20"/>
@@ -9536,29 +10349,81 @@
       <c r="K99" s="24"/>
       <c r="L99" s="27"/>
       <c r="M99" s="27"/>
+      <c r="N99" s="18"/>
+      <c r="O99" s="20"/>
+      <c r="P99" s="20"/>
+      <c r="Q99" s="20"/>
+      <c r="R99" s="20"/>
+      <c r="S99" s="20"/>
+      <c r="T99" s="20"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:K1"/>
   </mergeCells>
   <conditionalFormatting sqref="E3:E99">
-    <cfRule type="expression" dxfId="8" priority="1">
+    <cfRule type="expression" dxfId="8" priority="10">
       <formula>$D3="Fixed"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F3:H99">
-    <cfRule type="expression" dxfId="7" priority="2">
+  <conditionalFormatting sqref="F3:F99">
+    <cfRule type="expression" dxfId="7" priority="11">
+      <formula>OR($D3="Triangular",$D3="Beta-PERT",$D3="Uniform")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G3:G99">
+    <cfRule type="expression" dxfId="7" priority="12">
       <formula>OR($D3="Triangular",$D3="Beta-PERT")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I3:J99">
-    <cfRule type="expression" dxfId="6" priority="3">
-      <formula>$D3="Normal"</formula>
+  <conditionalFormatting sqref="H3:H99">
+    <cfRule type="expression" dxfId="7" priority="13">
+      <formula>OR($D3="Triangular",$D3="Beta-PERT",$D3="Uniform")</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="3">
+  <conditionalFormatting sqref="I3:I99">
+    <cfRule type="expression" dxfId="6" priority="14">
+      <formula>OR($D3="Normal",$D3="Exponential",$D3="Lognormal",$D3="Gamma")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J3:J99">
+    <cfRule type="expression" dxfId="6" priority="15">
+      <formula>OR($D3="Normal",$D3="Lognormal",$D3="Gamma")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="O3:O99">
+    <cfRule type="expression" dxfId="8" priority="16">
+      <formula>$N3="Fixed"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="P3:P99">
+    <cfRule type="expression" dxfId="7" priority="17">
+      <formula>OR($N3="Triangular",$N3="Beta-PERT",$N3="Uniform")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Q3:Q99">
+    <cfRule type="expression" dxfId="7" priority="18">
+      <formula>OR($N3="Triangular",$N3="Beta-PERT")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="R3:R99">
+    <cfRule type="expression" dxfId="7" priority="19">
+      <formula>OR($N3="Triangular",$N3="Beta-PERT",$N3="Uniform")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="S3:S99">
+    <cfRule type="expression" dxfId="6" priority="20">
+      <formula>OR($N3="Normal",$N3="Exponential",$N3="Lognormal",$N3="Gamma")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="T3:T99">
+    <cfRule type="expression" dxfId="6" priority="21">
+      <formula>OR($N3="Normal",$N3="Lognormal",$N3="Gamma")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="4">
     <dataValidation type="list" sqref="D3:D99" xr:uid="{00000000-0002-0000-0200-000000000000}">
-      <formula1>"Fixed,Triangular,Beta-PERT,Normal"</formula1>
+      <formula1>"Fixed,Triangular,Beta-PERT,Uniform,Normal,Exponential,Lognormal,Gamma"</formula1>
     </dataValidation>
     <dataValidation type="decimal" allowBlank="1" showErrorMessage="1" errorTitle="Invalid input" error="Enter a value from the documented options or range." sqref="K3:L99" xr:uid="{00000000-0002-0000-0200-000001000000}">
       <formula1>0</formula1>
@@ -9566,6 +10431,9 @@
     </dataValidation>
     <dataValidation type="list" showErrorMessage="1" error="Choose Fixed only or Fixed + time." sqref="M3:M99" xr:uid="{00000000-0002-0000-0200-000002000000}">
       <formula1>"Fixed only,Fixed + time"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" sqref="N3:N99">
+      <formula1>"Fixed,Triangular,Beta-PERT,Uniform,Normal,Exponential,Lognormal,Gamma"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -13720,7 +14588,7 @@
       <formula1>"Open,Monitoring,Closed"</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="N3:N99" xr:uid="{00000000-0002-0000-0300-000006000000}">
-      <formula1>"Fixed,Triangular,Beta-PERT,Normal"</formula1>
+      <formula1>"Fixed,Triangular,Beta-PERT,Uniform,Normal,Exponential,Lognormal,Gamma"</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="P3:P99" xr:uid="{00000000-0002-0000-0300-000007000000}">
       <formula1>"true,false"</formula1>
@@ -20085,28 +20953,33 @@
     <mergeCell ref="A1:J1"/>
   </mergeCells>
   <conditionalFormatting sqref="E3:E299">
-    <cfRule type="expression" dxfId="5" priority="1">
+    <cfRule type="expression" dxfId="5" priority="22">
       <formula>$D3="Fixed"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F3:F299">
-    <cfRule type="expression" dxfId="4" priority="2">
+    <cfRule type="expression" dxfId="4" priority="23">
       <formula>OR($D3="Triangular",$D3="Beta-PERT",$D3="Uniform")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G3:G299">
-    <cfRule type="expression" dxfId="3" priority="3">
+    <cfRule type="expression" dxfId="3" priority="24">
       <formula>OR($D3="Triangular",$D3="Beta-PERT")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H3:H299">
-    <cfRule type="expression" dxfId="2" priority="4">
+    <cfRule type="expression" dxfId="2" priority="25">
       <formula>OR($D3="Triangular",$D3="Beta-PERT",$D3="Uniform")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I3:J299">
-    <cfRule type="expression" dxfId="1" priority="5">
-      <formula>$D3="Normal"</formula>
+  <conditionalFormatting sqref="I3:I299">
+    <cfRule type="expression" dxfId="1" priority="26">
+      <formula>OR($D3="Normal",$D3="Exponential",$D3="Lognormal",$D3="Gamma")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J3:J299">
+    <cfRule type="expression" dxfId="1" priority="27">
+      <formula>OR($D3="Normal",$D3="Lognormal",$D3="Gamma")</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
@@ -20114,7 +20987,7 @@
       <formula1>"Duration,Cost"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Invalid input" error="Enter a value from the documented options or range." sqref="D3:D299" xr:uid="{00000000-0002-0000-0400-000001000000}">
-      <formula1>"Fixed,Triangular,Beta-PERT,Uniform,Normal"</formula1>
+      <formula1>"Fixed,Triangular,Beta-PERT,Uniform,Normal,Exponential,Lognormal,Gamma"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>